<commit_message>
Close to finalizing merge for GEM data
</commit_message>
<xml_diff>
--- a/Work/Data_Info/Meta_gem.xlsx
+++ b/Work/Data_Info/Meta_gem.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -390,6 +390,11 @@
           <t>var</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -422,6 +427,11 @@
           <t>Population</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -459,6 +469,11 @@
           <t>New.Housing.per.Capita</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -496,6 +511,11 @@
           <t>Permit.Housing.perCapita</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -533,6 +553,11 @@
           <t>Age.below.6</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -570,6 +595,11 @@
           <t>Age.6.18</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -607,6 +637,11 @@
           <t>Age.65</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -644,6 +679,11 @@
           <t>School.Primary</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -681,6 +721,11 @@
           <t>School.SpecialEdu</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -718,6 +763,11 @@
           <t>Migration.Balance</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -755,6 +805,11 @@
           <t>Purchasing.Power</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -792,6 +847,11 @@
           <t>Recreation.Area.per.Capita</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -829,6 +889,11 @@
           <t>Forest.Area</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -866,95 +931,110 @@
           <t>Water.Area</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Zuweisungen für Investitionsfördermaßnahmen in € je Einwohner</t>
+          <t>Einwohner je km²</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Zuweisungen für Investitionsfördermaßnahmen</t>
+          <t>Einwohnerdichte</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Zuweisungen für Investitionsfördermaßnahmen  &lt;Zeitpunkt&gt; / E &lt;Zeiitpunkt&gt;</t>
+          <t>E &lt;Zeitpunkt&gt; / Fläche &lt;Zeitpunkt&gt;</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Laufende Raumbeobachtung des BBSR; Vierteljährliche Kassenstatistik des Bundes und der Länder</t>
+          <t>Laufende Raumbeobachtung des BBSR; Fortschreibung des Bevölkerungsstandes des Bundes und der Länder</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Als Investitionszuweisungen bezeichnet man Finanztransfers von einer Einheit des öffentlichen Sektors an eine andere Einheit des öffentlichen Sektors (z.B. vom Land an eine Kommune). Die Finanztransfers dienen dabei der Investitionsfinanzierung. Investitionszuweisungen sind in der Bilanz des Zuweisungsempfängers bei den Sonderposten zu erfassen. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022.</t>
+          <t>Die Einwohnerdichte ist ein generelles Maß der regionalen Bevölkerungsverteilung und das am häufigsten verwendete Dichtemaß. Sie gibt Aufschluss zur Beurteilung des Arbeitsmarktes, der Auslastung von Infrastruktur, der Belastung der Umwelt usw. Zudem findet die Einwohnerdichte oft als zentraler Indikator Eingang in die Typisierung bzw. Differenzierung eher städtischer oder eher ländlicher Gebiete. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022.</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>9010</t>
+          <t>11004</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Investment.Allocations</t>
+          <t>Population.Density</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Einwohner je km²</t>
+          <t>Durchschn. Pkw-Fahrzeit zur nächsten BAB-Anschlussstelle in Minuten</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Einwohnerdichte</t>
+          <t>Erreichbarkeit von Autobahnen</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>E &lt;Zeitpunkt&gt; / Fläche &lt;Zeitpunkt&gt;</t>
+          <t>Pkw-Fahrzeit zur nächsten BAB-Anschlussstelle in Minuten &lt;Zeitpunkt&gt;</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Laufende Raumbeobachtung des BBSR; Fortschreibung des Bevölkerungsstandes des Bundes und der Länder</t>
+          <t>Laufende Raumbeobachtung des BBSR; Erreichbarkeitsmodell des BBSR</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Die Einwohnerdichte ist ein generelles Maß der regionalen Bevölkerungsverteilung und das am häufigsten verwendete Dichtemaß. Sie gibt Aufschluss zur Beurteilung des Arbeitsmarktes, der Auslastung von Infrastruktur, der Belastung der Umwelt usw. Zudem findet die Einwohnerdichte oft als zentraler Indikator Eingang in die Typisierung bzw. Differenzierung eher städtischer oder eher ländlicher Gebiete. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022.</t>
+          <t>Es handelt sich um den bevölkerungsgewichteten Durchschnittswert der auf der 100 m-Gitterzellenebene ermittelten Pkw-Fahrtzeiten zur zeitnächsten Bundesautobahnanschlussstelle. Die Erreichbarkeitsberechnungen des motorisierten Individualverkehrs basieren auf Routensuchen in einem Straßennetzmodell. Die Ermittlung der für Straßentypen zugrunde gelegten Pkw-Geschwindigkeiten erfolgt in Abhängigkeit von Ausbaustand sowie siedlungsstrukturellen und topographischen Gegebenheiten.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>11004</t>
+          <t>13101</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Population.Density</t>
+          <t>Highway.Access</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Durchschn. Pkw-Fahrzeit zur nächsten BAB-Anschlussstelle in Minuten</t>
+          <t>Durchschn. Pkw-Fahrzeit zum nächsten internationalen Flughafen in Deutschland in Minuten</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Erreichbarkeit von Autobahnen</t>
+          <t>Erreichbarkeit von Flughäfen</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pkw-Fahrzeit zur nächsten BAB-Anschlussstelle in Minuten &lt;Zeitpunkt&gt;</t>
+          <t>Pkw-Fahrzeit zum nächsten internationalen Flughafen in Minuten &lt;Zeitpunkt&gt;</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -964,34 +1044,39 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Es handelt sich um den bevölkerungsgewichteten Durchschnittswert der auf der 100 m-Gitterzellenebene ermittelten Pkw-Fahrtzeiten zur zeitnächsten Bundesautobahnanschlussstelle. Die Erreichbarkeitsberechnungen des motorisierten Individualverkehrs basieren auf Routensuchen in einem Straßennetzmodell. Die Ermittlung der für Straßentypen zugrunde gelegten Pkw-Geschwindigkeiten erfolgt in Abhängigkeit von Ausbaustand sowie siedlungsstrukturellen und topographischen Gegebenheiten.</t>
+          <t>Es handelt sich um den bevölkerungsgewichteten Durchschnittswert der auf der 100 m-Gitterzellenebene ermittelten Pkw-Fahrtzeiten zum zeitnächsten Hauptverkehrsflughafen in Deutschland oder dem benachbartem Ausland. Grundlage für die Auswahl der Flughäfen bildet die Luftverkehrsstatistik des Statistischen Bundesamtes sowie Daten des World Airport Traffic Report. Die Erreichbarkeitsberechnungen des motorisierten Individualverkehrs basieren auf Routensuchen in einem Straßennetzmodell. Die Ermittlung der für Straßentypen zugrunde gelegten Pkw-Geschwindigkeiten erfolgt in Abhängigkeit von Ausbaustand sowie siedlungsstrukturellen und topographischen Gegebenheiten.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>13101</t>
+          <t>13102</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Highway.Access</t>
+          <t>Airport.Access</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Durchschn. Pkw-Fahrzeit zum nächsten internationalen Flughafen in Deutschland in Minuten</t>
+          <t>Durchschn. Pkw-Fahrzeit zum nächsten IC/ICE-Bahnhof in Minuten</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Erreichbarkeit von Flughäfen</t>
+          <t>Erreichbarkeit von IC/EC/ICE-Bahnhöfen</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pkw-Fahrzeit zum nächsten internationalen Flughafen in Minuten &lt;Zeitpunkt&gt;</t>
+          <t>Pkw-Fahrzeit zum nächsten Bahnhof (Fernverkehr) in Minuten &lt;Zeitpunkt&gt;</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1001,108 +1086,123 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Es handelt sich um den bevölkerungsgewichteten Durchschnittswert der auf der 100 m-Gitterzellenebene ermittelten Pkw-Fahrtzeiten zum zeitnächsten Hauptverkehrsflughafen in Deutschland oder dem benachbartem Ausland. Grundlage für die Auswahl der Flughäfen bildet die Luftverkehrsstatistik des Statistischen Bundesamtes sowie Daten des World Airport Traffic Report. Die Erreichbarkeitsberechnungen des motorisierten Individualverkehrs basieren auf Routensuchen in einem Straßennetzmodell. Die Ermittlung der für Straßentypen zugrunde gelegten Pkw-Geschwindigkeiten erfolgt in Abhängigkeit von Ausbaustand sowie siedlungsstrukturellen und topographischen Gegebenheiten.</t>
+          <t>Es handelt sich um den bevölkerungsgewichteten Durchschnittswert der auf der 100 m-Gitterzelleneben ermittelten Pkw-Fahrtzeiten zum zeitnächsten IC-, EC- oder ICE-Haltepunkt. Bei den ausgewählten Bahnhöfen handelt es sich um alle IC-, EC- und ICE-Systemhalte der DB AG, selbst diejenigen in denen eine Bedienung nur durch einzelne Züge erfolgt. Die Erreichbarkeitsberechnungen des motorisierten Individualverkehrs basieren auf Routensuchen in einem Straßennetzmodell. Die Ermittlung der für Straßentypen zugrunde gelegten Pkw-Geschwindigkeiten erfolgt in Abhängigkeit von Ausbaustand sowie siedlungsstrukturellen und topographischen Gegebenheiten.</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>13102</t>
+          <t>13103</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Airport.Access</t>
+          <t>Highspeed.Rail.Access</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Durchschn. Pkw-Fahrzeit zum nächsten IC/ICE-Bahnhof in Minuten</t>
+          <t>Einwohnergewichtete Entfernung zum nächsten Supermarkt oder Discounter</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Erreichbarkeit von IC/EC/ICE-Bahnhöfen</t>
+          <t>Entfernung zum Supermarkt/Discounter</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pkw-Fahrzeit zum nächsten Bahnhof (Fernverkehr) in Minuten &lt;Zeitpunkt&gt;</t>
+          <t>Summe (Entfernung vom Messgittermittelpunkt zum nächsten Supermarkt/Discounter * Einwohnerzahl am Messpunktgitter) &lt;Zeitpunkt&gt; / Einwohner &lt;Zeitpunkt&gt;</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Laufende Raumbeobachtung des BBSR; Erreichbarkeitsmodell des BBSR</t>
+          <t>Laufende Raumbeobachtung des BBSR; POI Bund: BKG/GeoBasis-DE, infas360 GmbH; OSM Mitwirkende; Zensus 2022</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Es handelt sich um den bevölkerungsgewichteten Durchschnittswert der auf der 100 m-Gitterzelleneben ermittelten Pkw-Fahrtzeiten zum zeitnächsten IC-, EC- oder ICE-Haltepunkt. Bei den ausgewählten Bahnhöfen handelt es sich um alle IC-, EC- und ICE-Systemhalte der DB AG, selbst diejenigen in denen eine Bedienung nur durch einzelne Züge erfolgt. Die Erreichbarkeitsberechnungen des motorisierten Individualverkehrs basieren auf Routensuchen in einem Straßennetzmodell. Die Ermittlung der für Straßentypen zugrunde gelegten Pkw-Geschwindigkeiten erfolgt in Abhängigkeit von Ausbaustand sowie siedlungsstrukturellen und topographischen Gegebenheiten.</t>
+          <t>Indikator zur fußläufigen Erreichbarkeit des nächsten Supermarktes oder Discounter. Enthält die durchschnittliche, einwohnergewichtete Entfernung zum nächsten Supermarkt oder Discounter. Datengrundlage der Zielpunkte sind Standortdaten aus dem POI Bund Datensatz (Quelle: infas360 GmbH) sowie Ergänzungen aus OpenStreetMap (u.a. Nahversorger, Dorfläden, inhabergeführte Lebensmittelläden). Datengrundlage der Startpunkte sind Einwohnerzahlen des Zensus im 100x100m-Raster. Die Ermittlung der Distanzen erfolgt im 100x100m-Raster mit dem PathDistance-Algorithmus entlang von für Fußgänger passierbaren Wegesegmenten aus OpenStreetMap. Aufgrund wechselnder Datengrundlagen und Methoden der Distanzermittlung nicht für Zeitvergleiche geeignet.</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>13103</t>
+          <t>13106</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Highspeed.Rail.Access</t>
+          <t>Supermarket.Access</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Einwohnergewichtete Entfernung zum nächsten Supermarkt oder Discounter</t>
+          <t>Anteil Einwohner mit max. 1000m Entfernung zur nächsten Hausarztpraxis</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Entfernung zum Supermarkt/Discounter</t>
+          <t>Nahversorgung Hausarzt</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Summe (Entfernung vom Messgittermittelpunkt zum nächsten Supermarkt/Discounter * Einwohnerzahl am Messpunktgitter) &lt;Zeitpunkt&gt; / Einwohner &lt;Zeitpunkt&gt;</t>
+          <t>Einwohner mit max. 1km Entfernung zur nächsten Hausarztpraxis &lt;Zeitpunkt&gt; / Einwohner &lt;Zeitpunkt&gt; x 100</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Laufende Raumbeobachtung des BBSR; POI Bund: BKG/GeoBasis-DE, infas360 GmbH; OSM Mitwirkende; Zensus 2022</t>
+          <t>Laufende Raumbeobachtung des BBSR; POI Bund: BKG/GeoBasis-DE, infas360 GmbH; Zensus 2022</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Indikator zur fußläufigen Erreichbarkeit des nächsten Supermarktes oder Discounter. Enthält die durchschnittliche, einwohnergewichtete Entfernung zum nächsten Supermarkt oder Discounter. Datengrundlage der Zielpunkte sind Standortdaten aus dem POI Bund Datensatz (Quelle: infas360 GmbH) sowie Ergänzungen aus OpenStreetMap (u.a. Nahversorger, Dorfläden, inhabergeführte Lebensmittelläden). Datengrundlage der Startpunkte sind Einwohnerzahlen des Zensus im 100x100m-Raster. Die Ermittlung der Distanzen erfolgt im 100x100m-Raster mit dem PathDistance-Algorithmus entlang von für Fußgänger passierbaren Wegesegmenten aus OpenStreetMap. Aufgrund wechselnder Datengrundlagen und Methoden der Distanzermittlung nicht für Zeitvergleiche geeignet.</t>
+          <t>Indikator zur fußläufigen Erreichbarkeit der nächsten Hausarztpraxis. Enthält den Anteil der Einwohner mit einer Entfernung von max. 1000m zur nächsten Hausarztpraxis. Datengrundlage der Zielpunkte sind Standortdaten aus dem POI Bund Datensatz (Quelle: infas360 GmbH). Als Hausärzte sind definiert: Fachärzte für Allgemeinmedizin, Fachärzte für Innere und Allgemeinmedizin, Internisten, Praktische Ärzte ohne Schwerpunktbezeichnung. Datengrundlage der Startpunkte sind Einwohnerzahlen des Zensus im 100x100m-Raster. Die Ermittlung der Distanzen erfolgt im 100x100m-Raster mit dem PathDistance-Algorithmus entlang von für Fußgänger passierbaren Wegesegmenten aus OpenStreetMap. Aufgrund wechselnder Datengrundlagen und Methoden der Distanzermittlung nicht für Zeitvergleiche geeignet.</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>13106</t>
+          <t>13109</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Supermarket.Access</t>
+          <t>Doc.GP</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Anteil Einwohner mit max. 1000m Entfernung zur nächsten Hausarztpraxis</t>
+          <t>Einwohnergewichtete Entfernung zur nächsten Apotheke</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Nahversorgung Hausarzt</t>
+          <t>Entfernung zur Apotheke</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Einwohner mit max. 1km Entfernung zur nächsten Hausarztpraxis &lt;Zeitpunkt&gt; / Einwohner &lt;Zeitpunkt&gt; x 100</t>
+          <t>Summe (Entfernung vom Messgittermittelpunkt zur nächsten Apotheke * Einwohnerzahl am Messpunktgitter) &lt;Zeitpunkt&gt; / Einwohner &lt;Zeitpunkt&gt;</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1112,17 +1212,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Indikator zur fußläufigen Erreichbarkeit der nächsten Hausarztpraxis. Enthält den Anteil der Einwohner mit einer Entfernung von max. 1000m zur nächsten Hausarztpraxis. Datengrundlage der Zielpunkte sind Standortdaten aus dem POI Bund Datensatz (Quelle: infas360 GmbH). Als Hausärzte sind definiert: Fachärzte für Allgemeinmedizin, Fachärzte für Innere und Allgemeinmedizin, Internisten, Praktische Ärzte ohne Schwerpunktbezeichnung. Datengrundlage der Startpunkte sind Einwohnerzahlen des Zensus im 100x100m-Raster. Die Ermittlung der Distanzen erfolgt im 100x100m-Raster mit dem PathDistance-Algorithmus entlang von für Fußgänger passierbaren Wegesegmenten aus OpenStreetMap. Aufgrund wechselnder Datengrundlagen und Methoden der Distanzermittlung nicht für Zeitvergleiche geeignet.</t>
+          <t>Indikator zur fußläufigen Erreichbarkeit der nächsten Apotheke. Enthält die durchschnittliche, einwohnergewichtete Entfernung zur nächsten Apotheke. Datengrundlage der Zielpunkte sind Standortdaten aus dem POI Bund Datensatz (Quelle: infas360 GmbH). Datengrundlage der Startpunkte sind Einwohnerzahlen des Zensus im 100x100m-Raster. Die Ermittlung der Distanzen erfolgt im 100x100m-Raster mit dem PathDistance-Algorithmus entlang von für Fußgänger passierbaren Wegesegmenten aus OpenStreetMap. Aufgrund wechselnder Datengrundlagen und Methoden der Distanzermittlung nicht für Zeitvergleiche geeignet.</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>13109</t>
+          <t>13110</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
           <t>Pharmacy.Access</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
@@ -1165,6 +1270,11 @@
           <t>Broadband.50Mbps</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1205,6 +1315,11 @@
           <t>Broadband.100Mbps</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1245,206 +1360,236 @@
           <t>Broadband.1000Mbps</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>INKAR</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Anteil neu errichteter Ein- und Zweifamilienhäuser an den neu errichteten Häusern in %</t>
+          <t>Einwohnergewichtete Entfernung zur nächsten Haltestelle des ÖV mit mind. 20 Abfahrten am Tag</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Neue Ein- und Zweifamilienhäuser</t>
+          <t>Entfernung zur ÖV Haltestelle</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>fertiggestellte Wohngebäude mit 1 und 2 Wohnungen &lt;Zeitpunkt&gt; / fertiggestellte Wohngebäude &lt;Zeitpunkt&gt; x 100</t>
+          <t>Summe (Entfernung vom Messgittermittelpunkt zur nächsten ÖV-Haltestelle * Einwohnerzahl am Messpunktgitter) &lt;Zeitpunkt&gt; / Einwohner &lt;Zeitpunkt&gt;</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Laufende Raumbeobachtung des BBSR; Statistik der Baufertigstellungen des Bundes und der Länder</t>
+          <t>Laufende Raumbeobachtung des BBSR; Hacon Ingenieurgesellschaft mbH; Zensus 2022</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fertiggestellte Ein- und Zweifamilienhäuser sind ein indirekter Indikator für die Bautätigkeit im privat genutzten Wohneigentum. Durch den Bezug auf 'Gebäude im Bestand' wird die wohnungspolitische Bedeutung des Mehrfamilienhausbaus insbesondere in den Städten unterschätzt. Je nach gewünschter Aussage kannalternativ der Indikator 'Anteil Neubauwohnungen in Ein- und Zweifamilienhäusern' sinnvoll sein. </t>
+          <t>Indikator zur fußläufigen Erreichbarkeit der nächsten Haltestelle des ÖV. Enthält die durchschnittliche, einwohnergewichtete Entfernung zur nächsten Haltestelle des ÖV. Datengrundlage der Zielpunkte sind Haltestellen des öffentlichen Verkehrs aus einer Fahrplanabfrage (Quelle: Hacon Ingenieurgesellschaft mbH). Berücksichtigt wurden nur Haltestellen mit mind. 20 werktäglichen Abfahrten. Datengrundlage der Startpunkte sind Einwohnerzahlen des Zensus im 100x100m-Raster. Die Ermittlung der Distanzen erfolgt im 100x100m-Raster mit dem PathDistance-Algorithmus entlang von für Fußgänger passierbaren Wegesegmenten aus OpenStreetMap. Aufgrund wechselnder Datengrundlagen und Methoden der Distanzermittlung nicht für Zeitvergleiche geeignet.</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2106</t>
+          <t>13114</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>New.Family.Houses</t>
+          <t>Public.Transport.Access</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Einwohnergewichtete Entfernung zur nächsten Haltestelle des ÖV mit mind. 20 Abfahrten am Tag</t>
+          <t>Verunglückte im Straßenverkehr je 100.000 Einwohner</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Entfernung zur ÖV Haltestelle</t>
+          <t>Verunglückte im Straßenverkehr</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Summe (Entfernung vom Messgittermittelpunkt zur nächsten ÖV-Haltestelle * Einwohnerzahl am Messpunktgitter) &lt;Zeitpunkt&gt; / Einwohner &lt;Zeitpunkt&gt;</t>
+          <t>Verunglückte im Straßenverkehr &lt;Zeitpunkt&gt; / E &lt;Zeitpunkt&gt; x 100.000</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Laufende Raumbeobachtung des BBSR; Hacon Ingenieurgesellschaft mbH; Zensus 2022</t>
+          <t>Laufende Raumbeobachtung des BBSR; Statistik der Straßenverkehrsunfälle des Bundes und der Länder</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Indikator zur fußläufigen Erreichbarkeit der nächsten Haltestelle des ÖV. Enthält die durchschnittliche, einwohnergewichtete Entfernung zur nächsten Haltestelle des ÖV. Datengrundlage der Zielpunkte sind Haltestellen des öffentlichen Verkehrs aus einer Fahrplanabfrage (Quelle: Hacon Ingenieurgesellschaft mbH). Berücksichtigt wurden nur Haltestellen mit mind. 20 werktäglichen Abfahrten. Datengrundlage der Startpunkte sind Einwohnerzahlen des Zensus im 100x100m-Raster. Die Ermittlung der Distanzen erfolgt im 100x100m-Raster mit dem PathDistance-Algorithmus entlang von für Fußgänger passierbaren Wegesegmenten aus OpenStreetMap. Aufgrund wechselnder Datengrundlagen und Methoden der Distanzermittlung nicht für Zeitvergleiche geeignet.</t>
+          <t>Verunglückte sind Personen, die bei Unfällen infolge des Fahrverkehrs auf öffentlichen Wegen und Plätzen getötet oder verletzt wurden. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022.</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>13114</t>
+          <t>13211</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Public.Transport.Access</t>
+          <t>Traffic.Accidents</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Verunglückte im Straßenverkehr je 100.000 Einwohner</t>
+          <t>Nicht erwerbsfähige SGBII-Leistungsberechtigte unter 15 Jahren je 100 Einwohner unter 15 Jahren</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Verunglückte im Straßenverkehr</t>
+          <t>Kinderarmut</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Verunglückte im Straßenverkehr &lt;Zeitpunkt&gt; / E &lt;Zeitpunkt&gt; x 100.000</t>
+          <t>Nichterwerbsfähige Leistungsberechtigte unter 15 Jahren &lt;Zeitpunkt&gt; / Einwohner unter 15 Jahren &lt;Zeitpunkt&gt; x 100</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Laufende Raumbeobachtung des BBSR; Statistik der Straßenverkehrsunfälle des Bundes und der Länder</t>
+          <t>Laufende Raumbeobachtung des BBSR; Statistik der Grundsicherung für Arbeitsuchende der Bundesagentur für Arbeit</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Verunglückte sind Personen, die bei Unfällen infolge des Fahrverkehrs auf öffentlichen Wegen und Plätzen getötet oder verletzt wurden. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022.</t>
+          <t>Besonders betroffen von Kinderarmut sind Kinder Alleinerziehender sowie Kinder aus Familien mit ausländischer Herkunft oder aus Familien mit vielen Kindern. Der Indikator ist ein Hinweis auf deutlich schlechtere Zukunftschancen der entsprechenden Kinder. Die Grundsicherung für Arbeitsuchende nach dem SGB II soll die Absicherung des Existenzminimums, also die  Sicherung des zum Leben Notwendigen, sicherstellen. Diese Absicherung ist für alle gedacht, die zu wenig oder keine eigenen Mittel zur Verfügung haben. Es wird umgangssprachlich oft als 'Hartz IV' bezeichnet. Arbeitslosengeld II wird an erwerbsfähige Leistungsberechtigte gezahlt, Sozialgeld an nicht erwerbsfähige (Kinder unter 15 Jahren und Personen, die nicht arbeiten können). Trotz der Bezeichnung als Arbeitslosengeld ist Arbeitslosigkeit keine Voraussetzung, um Arbeitslosengeld II zu erhalten; es kann auch ergänzend zu anderem Einkommen und dem Arbeitslosengeld I bezogen werden. Erwerbsfähige Leistungsberechtigte (Empfänger von Arbeitslosengeld II) sind in der Lage mindestens 3 Stunden täglich unter den Bedingungen des allgemeinen Arbeitsmarktes tätig zu sein. Nicht erwerbsfähige Leistungsberechtigte (Empfänger von Sozialgeld) in einer Bedarfsgemeinschaft sind unter 15-Jährige oder Personen mit gesundheitlichen evtl. auch rechtlichen Einschränkungen, die nicht mindestens 3 Stunden täglich unter den allgemeinen Bedingungen arbeiten können. Ab dem Berichtsjahr 2016 wurde die Statistik umgestellt und der Personenkreis erweitert. Daher sind die Indikatoren bis 2015 und ab 2016 nur eingeschränkt miteinander vergleichbar. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022.</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>13211</t>
+          <t>12210</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Traffic.Accidents</t>
+          <t>Child.Poverty</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Nicht erwerbsfähige SGBII-Leistungsberechtigte unter 15 Jahren je 100 Einwohner unter 15 Jahren</t>
+          <t>Anzahl Kindertagesstätten</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Kinderarmut</t>
+          <t>Kindertagesstätten</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Nichterwerbsfähige Leistungsberechtigte unter 15 Jahren &lt;Zeitpunkt&gt; / Einwohner unter 15 Jahren &lt;Zeitpunkt&gt; x 100</t>
+          <t>Anzahl Kindertagesstätten</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Laufende Raumbeobachtung des BBSR; Statistik der Grundsicherung für Arbeitsuchende der Bundesagentur für Arbeit</t>
+          <t>Laufende Raumbeobachtung des BBSR; POI des BKG; Statistische Ämter der Länder und des Bundes</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Besonders betroffen von Kinderarmut sind Kinder Alleinerziehender sowie Kinder aus Familien mit ausländischer Herkunft oder aus Familien mit vielen Kindern. Der Indikator ist ein Hinweis auf deutlich schlechtere Zukunftschancen der entsprechenden Kinder. Die Grundsicherung für Arbeitsuchende nach dem SGB II soll die Absicherung des Existenzminimums, also die  Sicherung des zum Leben Notwendigen, sicherstellen. Diese Absicherung ist für alle gedacht, die zu wenig oder keine eigenen Mittel zur Verfügung haben. Es wird umgangssprachlich oft als 'Hartz IV' bezeichnet. Arbeitslosengeld II wird an erwerbsfähige Leistungsberechtigte gezahlt, Sozialgeld an nicht erwerbsfähige (Kinder unter 15 Jahren und Personen, die nicht arbeiten können). Trotz der Bezeichnung als Arbeitslosengeld ist Arbeitslosigkeit keine Voraussetzung, um Arbeitslosengeld II zu erhalten; es kann auch ergänzend zu anderem Einkommen und dem Arbeitslosengeld I bezogen werden. Erwerbsfähige Leistungsberechtigte (Empfänger von Arbeitslosengeld II) sind in der Lage mindestens 3 Stunden täglich unter den Bedingungen des allgemeinen Arbeitsmarktes tätig zu sein. Nicht erwerbsfähige Leistungsberechtigte (Empfänger von Sozialgeld) in einer Bedarfsgemeinschaft sind unter 15-Jährige oder Personen mit gesundheitlichen evtl. auch rechtlichen Einschränkungen, die nicht mindestens 3 Stunden täglich unter den allgemeinen Bedingungen arbeiten können. Ab dem Berichtsjahr 2016 wurde die Statistik umgestellt und der Personenkreis erweitert. Daher sind die Indikatoren bis 2015 und ab 2016 nur eingeschränkt miteinander vergleichbar. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022.</t>
+          <t>Es werden die Kindertageseinrichtungen erfasst, so wie sie von den jeweilig zuständigen Behörden erfasst werden. Es wird nur der Hauptstandort erfasst.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>12210</t>
+          <t>15631</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Child.Poverty</t>
+          <t>Daycare</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Anzahl Kindertagesstätten</t>
+          <t>SV Beschäftigte am Wohnort je 100 Einwohner im erwerbsfähigen Alter in %</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Kindertagesstätten</t>
+          <t>Beschäftigtenquote</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Anzahl Kindertagesstätten</t>
+          <t>SV Beschäftigte WO &lt;Zeitpunkt&gt; / E 15 bis &lt; 65 Jahre &lt;Zeitpunkt&gt; x 100</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Laufende Raumbeobachtung des BBSR; POI des BKG; Statistische Ämter der Länder und des Bundes</t>
+          <t>Laufende Raumbeobachtung des BBSR; Beschäftigtenstatistik der Bundesagentur für Arbeit</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Es werden die Kindertageseinrichtungen erfasst, so wie sie von den jeweilig zuständigen Behörden erfasst werden. Es wird nur der Hauptstandort erfasst.</t>
+          <t>Der Indikator bildet das Ausmaß der Beschäftigung bezogen auf alle Erwerbsfähigen ab. Konkret beschreibt er die Zahl sozialversicherungspflichtig Beschäftigter am Wohnort je 100 Einwohner im erwerbsfähigen Alter (15 bis unter 65 Jahre). Sozialversicherungspflichtig Beschäftigte sind Arbeiter, Angestellte und Personen in beruflicher Ausbildung, die in der gesetzlicher Renten-, Kranken- und/oder Arbeitslosenversicherung pflichtversichert sind. Keine Berücksichtigung finden hier also Beamte, Selbständige, mithelfende Familienangehörige oder geringfügig Beschäftigte. Insgesamt werden so nur rund 75% aller Erwerbstätigen erfasst. Trotz dieser Einschränkung werden die sozialversicherungspflichtig Beschäftigten als Maß der dem Arbeitsmarkt zur Verfügung stehenden Arbeitsplätze verwendet. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022. Bei den Beschäftigten handelt es sich um Zahlen zum Stichtag 30.06.. Ab 2013 handelt es sich um revidierte Daten (Revision 2014). Die Anzahl der sozialversicherungspflichtig Beschäftigten erhöhte sich dabei bundesweit um rund 350.000 Personen, das sind rund 1,2%.</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>15631</t>
+          <t>3101</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Daycare</t>
+          <t>Emp.Rate</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SV Beschäftigte am Wohnort je 100 Einwohner im erwerbsfähigen Alter in %</t>
+          <t>SV beschäftigte Frauen am Wohnort je 100 Frauen im erwerbsfähigen Alter in %</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Beschäftigtenquote</t>
+          <t>Beschäftigtenquote Frauen</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>SV Beschäftigte WO &lt;Zeitpunkt&gt; / E 15 bis &lt; 65 Jahre &lt;Zeitpunkt&gt; x 100</t>
+          <t>SV beschäftigte Frauen WO &lt;Zeitpunkt&gt; / weibl. E  15 bis &lt; 65 Jahre &lt;Zeitpunkt&gt; x 100</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1454,91 +1599,98 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Der Indikator bildet das Ausmaß der Beschäftigung bezogen auf alle Erwerbsfähigen ab. Konkret beschreibt er die Zahl sozialversicherungspflichtig Beschäftigter am Wohnort je 100 Einwohner im erwerbsfähigen Alter (15 bis unter 65 Jahre). Sozialversicherungspflichtig Beschäftigte sind Arbeiter, Angestellte und Personen in beruflicher Ausbildung, die in der gesetzlicher Renten-, Kranken- und/oder Arbeitslosenversicherung pflichtversichert sind. Keine Berücksichtigung finden hier also Beamte, Selbständige, mithelfende Familienangehörige oder geringfügig Beschäftigte. Insgesamt werden so nur rund 75% aller Erwerbstätigen erfasst. Trotz dieser Einschränkung werden die sozialversicherungspflichtig Beschäftigten als Maß der dem Arbeitsmarkt zur Verfügung stehenden Arbeitsplätze verwendet. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022. Bei den Beschäftigten handelt es sich um Zahlen zum Stichtag 30.06.. Ab 2013 handelt es sich um revidierte Daten (Revision 2014). Die Anzahl der sozialversicherungspflichtig Beschäftigten erhöhte sich dabei bundesweit um rund 350.000 Personen, das sind rund 1,2%.</t>
+          <t>Der Indikator bildet das Ausmaß der Beschäftigung von Frauen bezogen auf die Erwerbsfähigen dieser Bevölkerungsgruppe ab. Konkret beschreibt er die Zahl sozialversicherungspflichtig beschäftigter Frauen am Wohnort je 100 Frauen im erwerbsfähigen Alter (15 bis unter 65 Jahre). Sozialversicherungspflichtig Beschäftigte sind Arbeiter, Angestellte und Personen in beruflicher Ausbildung, die in der gesetzlicher Renten-, Kranken- und/oder Arbeitslosenversicherung pflichtversichert sind. Keine Berücksichtigung finden hier also Beamte, Selbständige, mithelfende Familienangehörige oder geringfügig Beschäftigte. Insgesamt werden so nur rund 75% aller Erwerbstätigen erfasst. Trotz dieser Einschränkung werden die sozialversicherungspflichtig Beschäftigten als Maß der dem Arbeitsmarkt zur Verfügung stehenden Arbeitsplätze verwendet. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022. Bei den Beschäftigten handelt es sich um Zahlen zum Stichtag 30.06..</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>3101</t>
+          <t>3102</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Emp.Rate</t>
+          <t>Emp.Rate.Women</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SV beschäftigte Frauen am Wohnort je 100 Frauen im erwerbsfähigen Alter in %</t>
+          <t>Anteil der arbeitslosen Männer an den Arbeitslosen in %</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Beschäftigtenquote Frauen</t>
+          <t>Arbeitslose Männer</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SV beschäftigte Frauen WO &lt;Zeitpunkt&gt; / weibl. E  15 bis &lt; 65 Jahre &lt;Zeitpunkt&gt; x 100</t>
+          <t>Arbeitslose Männer &lt;Zeitpunkt&gt; / Arbeitslose insgesamt &lt;Zeitpunkt&gt; x 100</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Laufende Raumbeobachtung des BBSR; Beschäftigtenstatistik der Bundesagentur für Arbeit</t>
+          <t>Laufende Raumbeobachtung des BBSR; Arbeitsmarktstatistik  der Bundesagentur für Arbeit (BA)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Der Indikator bildet das Ausmaß der Beschäftigung von Frauen bezogen auf die Erwerbsfähigen dieser Bevölkerungsgruppe ab. Konkret beschreibt er die Zahl sozialversicherungspflichtig beschäftigter Frauen am Wohnort je 100 Frauen im erwerbsfähigen Alter (15 bis unter 65 Jahre). Sozialversicherungspflichtig Beschäftigte sind Arbeiter, Angestellte und Personen in beruflicher Ausbildung, die in der gesetzlicher Renten-, Kranken- und/oder Arbeitslosenversicherung pflichtversichert sind. Keine Berücksichtigung finden hier also Beamte, Selbständige, mithelfende Familienangehörige oder geringfügig Beschäftigte. Insgesamt werden so nur rund 75% aller Erwerbstätigen erfasst. Trotz dieser Einschränkung werden die sozialversicherungspflichtig Beschäftigten als Maß der dem Arbeitsmarkt zur Verfügung stehenden Arbeitsplätze verwendet. Bei den Bevölkerungszahlen handelt es sich um die Fortschreibung des Bevölkerungsstandes des Bundes und der Länder zum Stichtag 31.12. des Jahres. Die Fortschreibung basiert auf der Volkszählung 1987 (BRD) bzw. 1981 (DDR), dem Zensus 2011 sowie dem Zensus 2022. Bei den Beschäftigten handelt es sich um Zahlen zum Stichtag 30.06..</t>
+          <t>Anteil der von Arbeitslosigkeit betroffenen Männer gegenüber der von Frauen. Männer haben ein höheres Risiko, ihre Beschäftigung zu verlieren und arbeitslos zu werden, aber auch bessere Chancen, Arbeitslosigkeit durch Aufnahme einer Beschäftigung wieder zu überwinden. Das liegt auch daran, dass Männer öfter in konjunktur- bzw. saisonabhängigen Berufen arbeiten.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>3102</t>
+          <t>1105</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Emp.Rate.Women</t>
+          <t>Unemp.Men</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>INKAR</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Anteil der arbeitslosen Männer an den Arbeitslosen in %</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Arbeitslose Männer</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Arbeitslose Männer &lt;Zeitpunkt&gt; / Arbeitslose insgesamt &lt;Zeitpunkt&gt; x 100</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Laufende Raumbeobachtung des BBSR; Arbeitsmarktstatistik  der Bundesagentur für Arbeit (BA)</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Anteil der von Arbeitslosigkeit betroffenen Männer gegenüber der von Frauen. Männer haben ein höheres Risiko, ihre Beschäftigung zu verlieren und arbeitslos zu werden, aber auch bessere Chancen, Arbeitslosigkeit durch Aufnahme einer Beschäftigung wieder zu überwinden. Das liegt auch daran, dass Männer öfter in konjunktur- bzw. saisonabhängigen Berufen arbeiten.</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>1105</t>
+          <t>Durchschnittliche Nettokaltmiete</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Unemp.Men</t>
+          <t>Rent.NetAvg</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Zensus 2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Durchschnittliche Nettokaltmiete</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Rent.NetAvg</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Zensus 2022</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
INKAR Data finalized for now
</commit_message>
<xml_diff>
--- a/Work/Data_Info/Meta_gem.xlsx
+++ b/Work/Data_Info/Meta_gem.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H33"/>
+  <dimension ref="A1:H32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -1677,23 +1677,6 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Durchschnittliche Nettokaltmiete</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>Rent.NetAvg</t>
-        </is>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Zensus 2022</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Mayor changes and extensions for index script(s)
</commit_message>
<xml_diff>
--- a/Work/Data_Info/Meta_gem.xlsx
+++ b/Work/Data_Info/Meta_gem.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>New.Housing.per.Capita</t>
+          <t>New_Housing_per_Capita</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -508,7 +508,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Permit.Housing.perCapita</t>
+          <t>Permit_Housing_perCapita</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Age.below.6</t>
+          <t>Age_below_6</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -592,7 +592,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Age.6.18</t>
+          <t>Age_6_18</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -634,7 +634,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Age.65</t>
+          <t>Age_65</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>School.Primary</t>
+          <t>School_Primary</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -718,7 +718,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>School.SpecialEdu</t>
+          <t>School_SpecialEdu</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Migration.Balance</t>
+          <t>Migration_Balance</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -802,7 +802,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Purchasing.Power</t>
+          <t>Purchasing_Power</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Recreation.Area.per.Capita</t>
+          <t>Recreation_Area_per_Capita</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -886,7 +886,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Forest.Area</t>
+          <t>Forest_Area</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -928,7 +928,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Water.Area</t>
+          <t>Water_Area</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Population.Density</t>
+          <t>Population_Density</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Highway.Access</t>
+          <t>Highway_Access</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Airport.Access</t>
+          <t>Airport_Access</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1096,7 +1096,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Highspeed.Rail.Access</t>
+          <t>Highspeed_Rail_Access</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Supermarket.Access</t>
+          <t>Supermarket_Access</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1180,7 +1180,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Doc.GP</t>
+          <t>Doc_GP</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1222,7 +1222,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Pharmacy.Access</t>
+          <t>Pharmacy_Access</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1267,7 +1267,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Broadband.50Mbps</t>
+          <t>Broadband_50Mbps</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Broadband.100Mbps</t>
+          <t>Broadband_100Mbps</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1357,7 +1357,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Broadband.1000Mbps</t>
+          <t>Broadband_1000Mbps</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Public.Transport.Access</t>
+          <t>Public_Transport_Access</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Traffic.Accidents</t>
+          <t>Traffic_Accidents</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Child.Poverty</t>
+          <t>Child_Poverty</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -1567,7 +1567,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Emp.Rate</t>
+          <t>Emp_Rate</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Emp.Rate.Women</t>
+          <t>Emp_Rate_Women</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Unemp.Men</t>
+          <t>Unemp_Men</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Rent.NetAvg</t>
+          <t>Rent_NetAvg</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">

</xml_diff>